<commit_message>
PVC pipe and motor options
</commit_message>
<xml_diff>
--- a/Information/Fan and motor options.xlsx
+++ b/Information/Fan and motor options.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/jdt57_cam_ac_uk/Documents/Engineering/IIA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\James\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{7443D3CF-E88C-4499-A106-8EB8E4F7A83B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0739887C-3592-4777-AD48-AA4367CBB4C7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77026C4C-DA6D-4910-AFAF-B0004402A5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{D14282AC-4677-4621-8D89-A06E360973EE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{D14282AC-4677-4621-8D89-A06E360973EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Rough Options" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="71">
   <si>
     <t>Motors &amp; Fans - SOLARSAFE</t>
   </si>
@@ -223,13 +223,37 @@
     <t>Total</t>
   </si>
   <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Dilwe Marine Bilge Blower,Quiet Strong 12V Ventilation Fan,4 Inch In Line Electric Air Blower for Yacht Boat Caravan RV : Amazon.co.uk: Sports &amp; Outdoors</t>
+  </si>
+  <si>
+    <t>2x T Junction, 2x 90deg turn/1x 180deg turn, length of straight section.</t>
+  </si>
+  <si>
+    <t>DHT11 Temperature-Humidity Sensor - The Pi Hut</t>
+  </si>
+  <si>
+    <t>ABX00033 | Arduino Nano Every with headers | RS</t>
+  </si>
+  <si>
+    <t>B&amp;Q</t>
+  </si>
+  <si>
+    <t>My basket at B&amp;Q</t>
+  </si>
+  <si>
     <t>amazon</t>
   </si>
   <si>
+    <t>https://www.amazon.co.uk/ALAMSCN-TEC1-12706-Thermoelectric-Cooling-Heatsink/dp/B0CBDH4BHL/ref=sr_1_10?dib=eyJ2IjoiMSJ9.SdjN396R8jWIR9UNV16f3FjYe6wEfqbM4VTd3OZxya46-BsiC508Cvbp-W2NH9kRH1AHTV4_HohK2f2J5JDMIInM4_B1VIxyQgeXTrW7Ws1v1NiXdnVxtBlGpzPblml3vPRAxfk9J2qIcsLjNHbv-Wwp4zByUXqiIPM2QB_7O0__uWtV0WrLrP3fCx-Itn2FyFC28WK0AxtsqIUvj-sKWga50ixVuRurcMACQI-v2JU.1wG4PdAXGVksMXwC9mfWs4XZp3xGZApFL-coIslo_xM&amp;dib_tag=se&amp;keywords=peltier+and+heatsink&amp;qid=1779714490&amp;sr=8-10</t>
+  </si>
+  <si>
     <t>https://www.amazon.co.uk/Heatsink-1-97x1-97x0-43-50mmx50mmx11mm-Amplifier-Transistor/dp/B0DPJTV3T1/ref=sr_1_3_sspa?dib=eyJ2IjoiMSJ9.SdjN396R8jWIR9UNV16f3FjYe6wEfqbM4VTd3OZxya46-BsiC508Cvbp-W2NH9kRH1AHTV4_HohK2f2J5JDMIInM4_B1VIxyQgeXTrW7Ws1v1NiXdnVxtBlGpzPblml3vPRAxfk9J2qIcsLjNHbv-Wwp4zByUXqiIPM2QB_7O0__uWtV0WrLrP3fCx-Itn2FyFC28WK0AxtsqIUvj-sKWga50ixVuRurcMACQI-v2JU.1wG4PdAXGVksMXwC9mfWs4XZp3xGZApFL-coIslo_xM&amp;dib_tag=se&amp;keywords=peltier+and+heatsink&amp;qid=1779714490&amp;sr=8-3-spons&amp;aref=6PFU1knfAE&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1</t>
-  </si>
-  <si>
-    <t>https://www.amazon.co.uk/ALAMSCN-TEC1-12706-Thermoelectric-Cooling-Heatsink/dp/B0CBDH4BHL/ref=sr_1_10?dib=eyJ2IjoiMSJ9.SdjN396R8jWIR9UNV16f3FjYe6wEfqbM4VTd3OZxya46-BsiC508Cvbp-W2NH9kRH1AHTV4_HohK2f2J5JDMIInM4_B1VIxyQgeXTrW7Ws1v1NiXdnVxtBlGpzPblml3vPRAxfk9J2qIcsLjNHbv-Wwp4zByUXqiIPM2QB_7O0__uWtV0WrLrP3fCx-Itn2FyFC28WK0AxtsqIUvj-sKWga50ixVuRurcMACQI-v2JU.1wG4PdAXGVksMXwC9mfWs4XZp3xGZApFL-coIslo_xM&amp;dib_tag=se&amp;keywords=peltier+and+heatsink&amp;qid=1779714490&amp;sr=8-10</t>
   </si>
 </sst>
 </file>
@@ -239,7 +263,7 @@
   <numFmts count="3">
     <numFmt numFmtId="6" formatCode="&quot;£&quot;#,##0;[Red]\-&quot;£&quot;#,##0"/>
     <numFmt numFmtId="8" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="174" formatCode="&quot;£&quot;#,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -274,7 +298,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -383,12 +407,56 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -399,24 +467,39 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -753,12 +836,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3A9A067-A91B-4EB3-BCFB-C152B07DAFBA}">
   <dimension ref="B2:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="7" max="7" width="8.21875" customWidth="1"/>
+    <col min="7" max="7" width="8.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
@@ -773,7 +856,7 @@
       </c>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>19</v>
       </c>
@@ -788,7 +871,7 @@
       </c>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B4" s="2" t="s">
         <v>20</v>
       </c>
@@ -803,7 +886,7 @@
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B5" s="2" t="s">
         <v>21</v>
       </c>
@@ -818,7 +901,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="2:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="58" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
@@ -841,18 +924,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0274B8E-02A6-4470-9501-7724AFEEBF2A}">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.77734375" customWidth="1"/>
-    <col min="10" max="10" width="159.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.81640625" customWidth="1"/>
+    <col min="10" max="10" width="159.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -860,35 +943,35 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B3" s="9" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="7"/>
-      <c r="J3" s="8" t="s">
+      <c r="I3" s="6"/>
+      <c r="J3" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B4" s="10" t="s">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B4" s="9" t="s">
         <v>3</v>
       </c>
       <c r="C4">
@@ -917,8 +1000,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B5" s="10" t="s">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B5" s="9" t="s">
         <v>4</v>
       </c>
       <c r="C5">
@@ -947,8 +1030,8 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B6" s="10" t="s">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B6" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C6">
@@ -977,8 +1060,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B7" s="10" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B7" s="9" t="s">
         <v>40</v>
       </c>
       <c r="C7">
@@ -1007,8 +1090,8 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B8" s="10" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B8" s="9" t="s">
         <v>42</v>
       </c>
       <c r="C8">
@@ -1037,8 +1120,8 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B9" s="11" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B9" s="10" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="5">
@@ -1063,7 +1146,7 @@
         <f t="shared" si="0"/>
         <v>2.3124999999999999E-3</v>
       </c>
-      <c r="J9" s="12" t="s">
+      <c r="J9" s="11" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1077,117 +1160,153 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{672EC7E8-D41F-4D53-A69D-327B6A7DDAE1}">
-  <dimension ref="B2:E11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:E11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B2" s="9" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B2" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="6" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="10" t="s">
+      <c r="E2" s="20" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="10" t="s">
+      <c r="C3" s="21">
+        <v>38.47</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B4" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="27">
         <v>8.9600000000000009</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="10" t="s">
+      <c r="D4" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="10" t="s">
+      <c r="C5" s="16">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B6" s="9" t="s">
         <v>50</v>
       </c>
       <c r="C6" s="17"/>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="10" t="s">
+      <c r="D6" s="14"/>
+      <c r="E6" s="4"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B7" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="30">
         <v>8.19</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B8" s="10" t="s">
+      <c r="D7" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B8" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="12">
         <f>2*3.9</f>
         <v>7.8</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="19" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" s="10" t="s">
+      <c r="E8" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B9" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="16"/>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B10" s="11" t="s">
+      <c r="C9" s="13"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="24"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B10" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="18">
         <v>13.31</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="5" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B11" s="9" t="s">
+      <c r="E10" s="23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B11" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="10">
         <f>SUM(C3:C10)</f>
-        <v>38.26</v>
-      </c>
-      <c r="D11" s="8"/>
+        <v>109.52999999999999</v>
+      </c>
+      <c r="D11" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="E3" r:id="rId1" display="https://www.amazon.co.uk/Marine-Blower-Electric-Ventilation-Caravan/dp/B0CT5LW2J1" xr:uid="{296B1FC8-93E0-433D-8A16-33B458E90078}"/>
+    <hyperlink ref="E8" r:id="rId2" display="https://thepihut.com/products/dht11-temperature-humidity-sensor" xr:uid="{9F451F42-CA4E-4840-9FBC-844A304DF836}"/>
+    <hyperlink ref="E10" r:id="rId3" display="https://uk.rs-online.com/web/p/arduino/1927590" xr:uid="{1C8F6D9E-BB32-48F4-859E-73C4E22917B7}"/>
+    <hyperlink ref="E5" r:id="rId4" display="https://www.diy.com/basket?redirectTo=%2Fdepartments%2Fmanrose-ducting-double-socket-44920-white-chrome-effect-push-fit-90-non-adjustable-bend-dia-100mm%2F5020953800736_BQ.prd" xr:uid="{EA444407-0D70-4AA7-968D-FCA160504202}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added electronics to parts list
</commit_message>
<xml_diff>
--- a/Information/Fan and motor options.xlsx
+++ b/Information/Fan and motor options.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\James\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zacheggie/Documents/Uni/Work/IIA/Eng for Poor Bill/2026-SolarSafe-Heating/Information/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77026C4C-DA6D-4910-AFAF-B0004402A5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B67604C1-E41A-D541-BF5C-29DB042625BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{D14282AC-4677-4621-8D89-A06E360973EE}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{D14282AC-4677-4621-8D89-A06E360973EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Rough Options" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="78">
   <si>
     <t>Motors &amp; Fans - SOLARSAFE</t>
   </si>
@@ -254,6 +254,27 @@
   </si>
   <si>
     <t>https://www.amazon.co.uk/Heatsink-1-97x1-97x0-43-50mmx50mmx11mm-Amplifier-Transistor/dp/B0DPJTV3T1/ref=sr_1_3_sspa?dib=eyJ2IjoiMSJ9.SdjN396R8jWIR9UNV16f3FjYe6wEfqbM4VTd3OZxya46-BsiC508Cvbp-W2NH9kRH1AHTV4_HohK2f2J5JDMIInM4_B1VIxyQgeXTrW7Ws1v1NiXdnVxtBlGpzPblml3vPRAxfk9J2qIcsLjNHbv-Wwp4zByUXqiIPM2QB_7O0__uWtV0WrLrP3fCx-Itn2FyFC28WK0AxtsqIUvj-sKWga50ixVuRurcMACQI-v2JU.1wG4PdAXGVksMXwC9mfWs4XZp3xGZApFL-coIslo_xM&amp;dib_tag=se&amp;keywords=peltier+and+heatsink&amp;qid=1779714490&amp;sr=8-3-spons&amp;aref=6PFU1knfAE&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1</t>
+  </si>
+  <si>
+    <t>Bread board</t>
+  </si>
+  <si>
+    <t>Jumper wires</t>
+  </si>
+  <si>
+    <t>USB micro-b / micro USB (depending on model of arduino)</t>
+  </si>
+  <si>
+    <t>Misc passives</t>
+  </si>
+  <si>
+    <t>Misc. Electronics</t>
+  </si>
+  <si>
+    <t>Motor driver</t>
+  </si>
+  <si>
+    <t>https://www.amazon.co.uk/JZK-BTS7960B-Double-Stepper-H-Bridge/dp/B09HGBM5D2</t>
   </si>
 </sst>
 </file>
@@ -261,9 +282,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="6" formatCode="&quot;£&quot;#,##0;[Red]\-&quot;£&quot;#,##0"/>
-    <numFmt numFmtId="8" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
-    <numFmt numFmtId="174" formatCode="&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0;[Red]\-&quot;£&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="&quot;£&quot;#,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -456,7 +477,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -473,33 +494,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyBorder="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -836,12 +852,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3A9A067-A91B-4EB3-BCFB-C152B07DAFBA}">
   <dimension ref="B2:G6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="7" max="7" width="8.1796875" customWidth="1"/>
+    <col min="7" max="7" width="8.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:7" ht="32" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
@@ -856,7 +872,7 @@
       </c>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:7" ht="32" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
         <v>19</v>
       </c>
@@ -871,7 +887,7 @@
       </c>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:7" ht="32" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
         <v>20</v>
       </c>
@@ -886,7 +902,7 @@
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="2:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:7" ht="48" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
         <v>21</v>
       </c>
@@ -901,7 +917,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="2:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:7" ht="64" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
@@ -924,18 +940,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0274B8E-02A6-4470-9501-7724AFEEBF2A}">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.81640625" customWidth="1"/>
-    <col min="10" max="10" width="159.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="159.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -943,7 +959,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B3" s="8" t="s">
         <v>1</v>
       </c>
@@ -970,7 +986,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B4" s="9" t="s">
         <v>3</v>
       </c>
@@ -1000,7 +1016,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B5" s="9" t="s">
         <v>4</v>
       </c>
@@ -1030,7 +1046,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B6" s="9" t="s">
         <v>31</v>
       </c>
@@ -1060,7 +1076,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B7" s="9" t="s">
         <v>40</v>
       </c>
@@ -1090,7 +1106,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B8" s="9" t="s">
         <v>42</v>
       </c>
@@ -1120,7 +1136,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>5</v>
       </c>
@@ -1160,140 +1176,177 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{672EC7E8-D41F-4D53-A69D-327B6A7DDAE1}">
-  <dimension ref="A2:E11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A2:E19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="57.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B2" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="12" t="s">
         <v>55</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="21">
+      <c r="C3" s="16">
         <v>38.47</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="18" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B4" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="27">
+      <c r="C4" s="19">
         <v>8.9600000000000009</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>63</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="13">
         <v>32.799999999999997</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="18" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B6" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="14"/>
+      <c r="C6" s="14"/>
       <c r="E6" s="4"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B7" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C7" s="30">
+      <c r="C7" s="19">
         <v>8.19</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="28" t="s">
+      <c r="E7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B8" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="20">
         <f>2*3.9</f>
         <v>7.8</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="23" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B9" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="24"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C9" s="21"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B10" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="15">
         <v>13.31</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="E10" s="18" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B11" s="8" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B11" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="15">
+        <v>7.19</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B12" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="10">
-        <f>SUM(C3:C10)</f>
-        <v>109.52999999999999</v>
-      </c>
-      <c r="D11" s="14"/>
+      <c r="C12" s="25">
+        <f>SUM(C3:C11)</f>
+        <v>116.71999999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>74</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>